<commit_message>
fix: 8 bugs - JS null checks, listener leak, api keuangan, CPO alert, create_excel header
</commit_message>
<xml_diff>
--- a/data/harga_emas.xlsx
+++ b/data/harga_emas.xlsx
@@ -1422,7 +1422,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N66"/>
+  <dimension ref="A1:N97"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -4630,6 +4630,1494 @@
         <v>0</v>
       </c>
       <c r="N66" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
+      <c r="B67" s="2" t="inlineStr">
+        <is>
+          <t>Antam</t>
+        </is>
+      </c>
+      <c r="C67" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="D67" s="3" t="n">
+        <v>2673000</v>
+      </c>
+      <c r="E67" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F67" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G67" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H67" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I67" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="J67" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="K67" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="L67" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M67" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="N67" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
+      <c r="B68" s="2" t="inlineStr">
+        <is>
+          <t>Antam</t>
+        </is>
+      </c>
+      <c r="C68" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="D68" s="3" t="n">
+        <v>2673000</v>
+      </c>
+      <c r="E68" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F68" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G68" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H68" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I68" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="J68" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="K68" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="L68" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M68" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="N68" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
+      <c r="B69" s="2" t="inlineStr">
+        <is>
+          <t>Antam</t>
+        </is>
+      </c>
+      <c r="C69" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="D69" s="3" t="n">
+        <v>2673000</v>
+      </c>
+      <c r="E69" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F69" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G69" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H69" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I69" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="J69" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="K69" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="L69" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M69" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="N69" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
+      <c r="B70" s="2" t="inlineStr">
+        <is>
+          <t>Antam</t>
+        </is>
+      </c>
+      <c r="C70" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="D70" s="3" t="n">
+        <v>2673000</v>
+      </c>
+      <c r="E70" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F70" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G70" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H70" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I70" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="J70" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="K70" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="L70" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M70" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="N70" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
+      <c r="B71" s="2" t="inlineStr">
+        <is>
+          <t>Antam</t>
+        </is>
+      </c>
+      <c r="C71" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="D71" s="3" t="n">
+        <v>2673000</v>
+      </c>
+      <c r="E71" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F71" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G71" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H71" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I71" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="J71" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="K71" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="L71" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M71" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="N71" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
+      <c r="B72" s="2" t="inlineStr">
+        <is>
+          <t>Antam</t>
+        </is>
+      </c>
+      <c r="C72" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="D72" s="3" t="n">
+        <v>2673000</v>
+      </c>
+      <c r="E72" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F72" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G72" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H72" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I72" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="J72" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="K72" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="L72" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M72" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="N72" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
+      <c r="B73" s="2" t="inlineStr">
+        <is>
+          <t>Antam</t>
+        </is>
+      </c>
+      <c r="C73" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="D73" s="3" t="n">
+        <v>2673000</v>
+      </c>
+      <c r="E73" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F73" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G73" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H73" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I73" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="J73" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="K73" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="L73" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M73" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="N73" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
+      <c r="B74" s="2" t="inlineStr">
+        <is>
+          <t>Antam</t>
+        </is>
+      </c>
+      <c r="C74" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="D74" s="3" t="n">
+        <v>2673000</v>
+      </c>
+      <c r="E74" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F74" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G74" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H74" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I74" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="J74" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="K74" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="L74" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M74" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="N74" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
+      <c r="B75" s="2" t="inlineStr">
+        <is>
+          <t>Antam</t>
+        </is>
+      </c>
+      <c r="C75" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="D75" s="3" t="n">
+        <v>2673000</v>
+      </c>
+      <c r="E75" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F75" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G75" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H75" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I75" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="J75" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="K75" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="L75" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M75" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="N75" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
+      <c r="B76" s="2" t="inlineStr">
+        <is>
+          <t>Antam</t>
+        </is>
+      </c>
+      <c r="C76" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="D76" s="3" t="n">
+        <v>2673000</v>
+      </c>
+      <c r="E76" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F76" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G76" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H76" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I76" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="J76" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="K76" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="L76" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M76" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="N76" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
+      <c r="B77" s="2" t="inlineStr">
+        <is>
+          <t>Antam</t>
+        </is>
+      </c>
+      <c r="C77" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="D77" s="3" t="n">
+        <v>2673000</v>
+      </c>
+      <c r="E77" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F77" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G77" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H77" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I77" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="J77" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="K77" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="L77" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M77" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="N77" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
+      <c r="B78" s="2" t="inlineStr">
+        <is>
+          <t>Antam</t>
+        </is>
+      </c>
+      <c r="C78" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="D78" s="3" t="n">
+        <v>2673000</v>
+      </c>
+      <c r="E78" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F78" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G78" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H78" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I78" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="J78" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="K78" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="L78" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M78" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="N78" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
+      <c r="B79" s="2" t="inlineStr">
+        <is>
+          <t>Antam</t>
+        </is>
+      </c>
+      <c r="C79" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="D79" s="3" t="n">
+        <v>2673000</v>
+      </c>
+      <c r="E79" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F79" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G79" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H79" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I79" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="J79" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="K79" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="L79" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M79" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="N79" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
+      <c r="B80" s="2" t="inlineStr">
+        <is>
+          <t>Antam</t>
+        </is>
+      </c>
+      <c r="C80" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="D80" s="3" t="n">
+        <v>2673000</v>
+      </c>
+      <c r="E80" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F80" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G80" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H80" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I80" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="J80" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="K80" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="L80" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M80" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="N80" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
+      <c r="B81" s="2" t="inlineStr">
+        <is>
+          <t>Antam</t>
+        </is>
+      </c>
+      <c r="C81" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="D81" s="3" t="n">
+        <v>2673000</v>
+      </c>
+      <c r="E81" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F81" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G81" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H81" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I81" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="J81" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="K81" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="L81" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M81" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="N81" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
+      <c r="B82" s="2" t="inlineStr">
+        <is>
+          <t>Antam</t>
+        </is>
+      </c>
+      <c r="C82" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="D82" s="3" t="n">
+        <v>2673000</v>
+      </c>
+      <c r="E82" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F82" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G82" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H82" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I82" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="J82" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="K82" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="L82" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M82" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="N82" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
+      <c r="B83" s="2" t="inlineStr">
+        <is>
+          <t>Antam</t>
+        </is>
+      </c>
+      <c r="C83" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="D83" s="3" t="n">
+        <v>2673000</v>
+      </c>
+      <c r="E83" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F83" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G83" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H83" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I83" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="J83" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="K83" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="L83" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M83" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="N83" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
+      <c r="B84" s="2" t="inlineStr">
+        <is>
+          <t>Antam</t>
+        </is>
+      </c>
+      <c r="C84" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="D84" s="3" t="n">
+        <v>2673000</v>
+      </c>
+      <c r="E84" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F84" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G84" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H84" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I84" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="J84" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="K84" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="L84" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M84" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="N84" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
+      <c r="B85" s="2" t="inlineStr">
+        <is>
+          <t>Antam</t>
+        </is>
+      </c>
+      <c r="C85" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="D85" s="3" t="n">
+        <v>2673000</v>
+      </c>
+      <c r="E85" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F85" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G85" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H85" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I85" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="J85" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="K85" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="L85" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M85" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="N85" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
+      <c r="B86" s="2" t="inlineStr">
+        <is>
+          <t>Antam</t>
+        </is>
+      </c>
+      <c r="C86" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="D86" s="3" t="n">
+        <v>2673000</v>
+      </c>
+      <c r="E86" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F86" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G86" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H86" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I86" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="J86" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="K86" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="L86" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M86" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="N86" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
+      <c r="B87" s="2" t="inlineStr">
+        <is>
+          <t>Antam</t>
+        </is>
+      </c>
+      <c r="C87" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="D87" s="3" t="n">
+        <v>2673000</v>
+      </c>
+      <c r="E87" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F87" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G87" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H87" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I87" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="J87" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="K87" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="L87" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M87" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="N87" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
+      <c r="B88" s="2" t="inlineStr">
+        <is>
+          <t>Antam</t>
+        </is>
+      </c>
+      <c r="C88" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="D88" s="3" t="n">
+        <v>2673000</v>
+      </c>
+      <c r="E88" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F88" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G88" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H88" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I88" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="J88" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="K88" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="L88" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M88" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="N88" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
+      <c r="B89" s="2" t="inlineStr">
+        <is>
+          <t>Antam</t>
+        </is>
+      </c>
+      <c r="C89" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="D89" s="3" t="n">
+        <v>2673000</v>
+      </c>
+      <c r="E89" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F89" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G89" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H89" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I89" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="J89" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="K89" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="L89" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M89" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="N89" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
+      <c r="B90" s="2" t="inlineStr">
+        <is>
+          <t>Antam</t>
+        </is>
+      </c>
+      <c r="C90" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="D90" s="3" t="n">
+        <v>2673000</v>
+      </c>
+      <c r="E90" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F90" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G90" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H90" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I90" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="J90" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="K90" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="L90" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M90" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="N90" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
+      <c r="B91" s="2" t="inlineStr">
+        <is>
+          <t>Antam</t>
+        </is>
+      </c>
+      <c r="C91" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="D91" s="3" t="n">
+        <v>2673000</v>
+      </c>
+      <c r="E91" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F91" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G91" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H91" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I91" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="J91" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="K91" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="L91" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M91" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="N91" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
+      <c r="B92" s="2" t="inlineStr">
+        <is>
+          <t>Antam</t>
+        </is>
+      </c>
+      <c r="C92" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="D92" s="3" t="n">
+        <v>2673000</v>
+      </c>
+      <c r="E92" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F92" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G92" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H92" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I92" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="J92" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="K92" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="L92" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M92" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="N92" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
+      <c r="B93" s="2" t="inlineStr">
+        <is>
+          <t>Antam</t>
+        </is>
+      </c>
+      <c r="C93" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="D93" s="3" t="n">
+        <v>2673000</v>
+      </c>
+      <c r="E93" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F93" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G93" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H93" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I93" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="J93" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="K93" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="L93" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M93" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="N93" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
+      <c r="B94" s="2" t="inlineStr">
+        <is>
+          <t>Antam</t>
+        </is>
+      </c>
+      <c r="C94" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="D94" s="3" t="n">
+        <v>2673000</v>
+      </c>
+      <c r="E94" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F94" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G94" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H94" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I94" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="J94" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="K94" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="L94" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M94" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="N94" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
+      <c r="B95" s="2" t="inlineStr">
+        <is>
+          <t>Antam</t>
+        </is>
+      </c>
+      <c r="C95" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="D95" s="3" t="n">
+        <v>2673000</v>
+      </c>
+      <c r="E95" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F95" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G95" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H95" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I95" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="J95" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="K95" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="L95" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M95" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="N95" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
+      <c r="B96" s="2" t="inlineStr">
+        <is>
+          <t>Antam</t>
+        </is>
+      </c>
+      <c r="C96" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="D96" s="3" t="n">
+        <v>2673000</v>
+      </c>
+      <c r="E96" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F96" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G96" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H96" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I96" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="J96" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="K96" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="L96" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M96" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="N96" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
+      <c r="B97" s="2" t="inlineStr">
+        <is>
+          <t>Antam</t>
+        </is>
+      </c>
+      <c r="C97" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="D97" s="3" t="n">
+        <v>2673000</v>
+      </c>
+      <c r="E97" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F97" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G97" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H97" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I97" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="J97" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="K97" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="L97" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M97" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="N97" s="2" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>